<commit_message>
class room observation form added
</commit_message>
<xml_diff>
--- a/Sindhi Muslim/New Admissions 2025-2026/Student Registration.xlsx
+++ b/Sindhi Muslim/New Admissions 2025-2026/Student Registration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Government-High-School\Sindhi Muslim\New Admissions 2025-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4BC992F-EE1E-47C0-8977-407185790E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD03E1F-D1EE-4043-8E2D-7597E37B91E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{8EEF71F7-8EBE-4B4E-97F3-3DF7586E05F6}"/>
+    <workbookView xWindow="30" yWindow="30" windowWidth="20460" windowHeight="10890" xr2:uid="{8EEF71F7-8EBE-4B4E-97F3-3DF7586E05F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Registration" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="153">
   <si>
     <t>S No</t>
   </si>
@@ -493,6 +493,12 @@
   </si>
   <si>
     <t>Pending</t>
+  </si>
+  <si>
+    <t>Ariyan Khan</t>
+  </si>
+  <si>
+    <t>Muhammad Ismail</t>
   </si>
 </sst>
 </file>
@@ -746,12 +752,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -760,6 +760,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1092,6 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1828FFCB-D8F5-4B91-AACC-9381EDE31E0A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1135,7 +1142,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1164,7 +1171,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1249,7 +1256,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1303,7 +1310,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1330,7 +1337,7 @@
       </c>
       <c r="I8" s="6"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1357,7 +1364,7 @@
       </c>
       <c r="I9" s="6"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1382,7 +1389,7 @@
       </c>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1409,7 +1416,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1434,7 +1441,7 @@
       </c>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1463,7 +1470,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1490,7 +1497,7 @@
       </c>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1515,7 +1522,7 @@
       </c>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1540,7 +1547,7 @@
       </c>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1569,7 +1576,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1594,7 +1601,7 @@
       </c>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1619,7 +1626,7 @@
       </c>
       <c r="I19" s="6"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1644,7 +1651,7 @@
       </c>
       <c r="I20" s="6"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1669,7 +1676,7 @@
       </c>
       <c r="I21" s="6"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1698,7 +1705,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1725,7 +1732,7 @@
       </c>
       <c r="I23" s="6"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1750,7 +1757,7 @@
       </c>
       <c r="I24" s="6"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1775,7 +1782,7 @@
       </c>
       <c r="I25" s="6"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1804,7 +1811,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1831,7 +1838,7 @@
       </c>
       <c r="I27" s="6"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1856,7 +1863,7 @@
       </c>
       <c r="I28" s="6"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1883,7 +1890,7 @@
       </c>
       <c r="I29" s="6"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1910,7 +1917,7 @@
       </c>
       <c r="I30" s="6"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -1935,7 +1942,7 @@
       </c>
       <c r="I31" s="6"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1962,7 +1969,7 @@
       </c>
       <c r="I32" s="6"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -1991,7 +1998,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2018,7 +2025,7 @@
       </c>
       <c r="I34" s="6"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2043,7 +2050,7 @@
       </c>
       <c r="I35" s="6"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2066,7 +2073,7 @@
       </c>
       <c r="I36" s="6"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2091,7 +2098,7 @@
       </c>
       <c r="I37" s="6"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2118,7 +2125,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2143,7 +2150,7 @@
       </c>
       <c r="I39" s="6"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2172,7 +2179,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2197,7 +2204,7 @@
       </c>
       <c r="I41" s="6"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2222,7 +2229,7 @@
       </c>
       <c r="I42" s="6"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2330,7 +2337,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2357,7 +2364,7 @@
       </c>
       <c r="I47" s="6"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2380,7 +2387,7 @@
       </c>
       <c r="I48" s="6"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2403,7 +2410,7 @@
       </c>
       <c r="I49" s="6"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2432,7 +2439,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2459,7 +2466,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2551,18 +2558,30 @@
       <c r="A55" s="2">
         <v>54</v>
       </c>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
+      <c r="B55" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="E55" s="3"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="I55" s="6"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F55" s="4">
+        <v>3053196212</v>
+      </c>
+      <c r="G55" s="5">
+        <v>45764</v>
+      </c>
+      <c r="H55" s="5">
+        <v>45766</v>
+      </c>
+      <c r="I55" s="6">
+        <v>0.4375</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2577,7 +2596,7 @@
       </c>
       <c r="I56" s="6"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2592,7 +2611,7 @@
       </c>
       <c r="I57" s="6"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2607,7 +2626,7 @@
       </c>
       <c r="I58" s="6"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2622,7 +2641,7 @@
       </c>
       <c r="I59" s="6"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2637,7 +2656,7 @@
       </c>
       <c r="I60" s="6"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2652,7 +2671,7 @@
       </c>
       <c r="I61" s="6"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2667,7 +2686,7 @@
       </c>
       <c r="I62" s="6"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2682,7 +2701,7 @@
       </c>
       <c r="I63" s="6"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2697,7 +2716,7 @@
       </c>
       <c r="I64" s="6"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2712,7 +2731,7 @@
       </c>
       <c r="I65" s="6"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2727,7 +2746,7 @@
       </c>
       <c r="I66" s="6"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2742,7 +2761,7 @@
       </c>
       <c r="I67" s="6"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2757,7 +2776,7 @@
       </c>
       <c r="I68" s="6"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2772,7 +2791,7 @@
       </c>
       <c r="I69" s="6"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2787,7 +2806,7 @@
       </c>
       <c r="I70" s="6"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2802,7 +2821,7 @@
       </c>
       <c r="I71" s="6"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2817,7 +2836,7 @@
       </c>
       <c r="I72" s="6"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -2832,7 +2851,7 @@
       </c>
       <c r="I73" s="6"/>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -2847,7 +2866,7 @@
       </c>
       <c r="I74" s="6"/>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -2862,7 +2881,7 @@
       </c>
       <c r="I75" s="6"/>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -2877,7 +2896,7 @@
       </c>
       <c r="I76" s="6"/>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -2892,7 +2911,7 @@
       </c>
       <c r="I77" s="6"/>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -2907,7 +2926,7 @@
       </c>
       <c r="I78" s="6"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -2922,7 +2941,7 @@
       </c>
       <c r="I79" s="6"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -2937,7 +2956,7 @@
       </c>
       <c r="I80" s="6"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -2952,7 +2971,7 @@
       </c>
       <c r="I81" s="6"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -2967,7 +2986,7 @@
       </c>
       <c r="I82" s="6"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -2982,7 +3001,7 @@
       </c>
       <c r="I83" s="6"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -2997,7 +3016,7 @@
       </c>
       <c r="I84" s="6"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3012,7 +3031,7 @@
       </c>
       <c r="I85" s="6"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3027,7 +3046,7 @@
       </c>
       <c r="I86" s="6"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3042,7 +3061,7 @@
       </c>
       <c r="I87" s="6"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3057,7 +3076,7 @@
       </c>
       <c r="I88" s="6"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3072,7 +3091,7 @@
       </c>
       <c r="I89" s="6"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3087,7 +3106,7 @@
       </c>
       <c r="I90" s="6"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3102,7 +3121,7 @@
       </c>
       <c r="I91" s="6"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3118,7 +3137,13 @@
       <c r="I92" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I92" xr:uid="{1828FFCB-D8F5-4B91-AACC-9381EDE31E0A}"/>
+  <autoFilter ref="A1:I92" xr:uid="{1828FFCB-D8F5-4B91-AACC-9381EDE31E0A}">
+    <filterColumn colId="7">
+      <filters>
+        <dateGroupItem year="2025" month="4" day="19" dateTimeGrouping="day"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A1:I92">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$H1&lt;TODAY()</formula>
@@ -3436,13 +3461,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="20"/>
     </row>
     <row r="2" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -3493,20 +3518,20 @@
       <c r="A7" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="19"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="22"/>
     </row>
     <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="22"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20"/>
     </row>
     <row r="22" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
@@ -3557,19 +3582,13 @@
       <c r="A27" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B7:E7"/>
@@ -3578,6 +3597,12 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>